<commit_message>
Implement import, breakbulk, testing, and UI refinements
</commit_message>
<xml_diff>
--- a/docs/templates/veiculos-modelo.xlsx
+++ b/docs/templates/veiculos-modelo.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="Modelo" sheetId="1" r:id="rId1"/>
+    <sheet name="VEICULOS" sheetId="1" r:id="rId1"/>
   </sheets>
 </workbook>
 </file>
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H3"/>
+  <dimension ref="A1:I3"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -407,21 +407,24 @@
         <v>MARCA</v>
       </c>
       <c r="C1" t="str">
+        <v>MODELO</v>
+      </c>
+      <c r="D1" t="str">
         <v>PESO</v>
       </c>
-      <c r="D1" t="str">
+      <c r="E1" t="str">
         <v>CUBAGEM</v>
       </c>
-      <c r="E1" t="str">
+      <c r="F1" t="str">
         <v>CONTAINER</v>
       </c>
-      <c r="F1" t="str">
+      <c r="G1" t="str">
         <v>TIPO_CONTAINER</v>
       </c>
-      <c r="G1" t="str">
+      <c r="H1" t="str">
         <v>LACRE</v>
       </c>
-      <c r="H1" t="str">
+      <c r="I1" t="str">
         <v>BL</v>
       </c>
     </row>
@@ -432,22 +435,25 @@
       <c r="B2" t="str">
         <v>VOLKSWAGEN</v>
       </c>
-      <c r="C2">
+      <c r="C2" t="str">
+        <v>NIVUS</v>
+      </c>
+      <c r="D2">
         <v>1320</v>
       </c>
-      <c r="D2">
+      <c r="E2">
         <v>8.75</v>
       </c>
-      <c r="E2" t="str">
+      <c r="F2" t="str">
         <v>TEMU1234567</v>
       </c>
-      <c r="F2" t="str">
+      <c r="G2" t="str">
         <v>40HC</v>
       </c>
-      <c r="G2" t="str">
+      <c r="H2" t="str">
         <v>SEAL001</v>
       </c>
-      <c r="H2" t="str">
+      <c r="I2" t="str">
         <v>BL12345678</v>
       </c>
     </row>
@@ -458,28 +464,31 @@
       <c r="B3" t="str">
         <v>PEUGEOT</v>
       </c>
-      <c r="C3">
+      <c r="C3" t="str">
+        <v>2008</v>
+      </c>
+      <c r="D3">
         <v>1290</v>
       </c>
-      <c r="D3">
+      <c r="E3">
         <v>8.1</v>
       </c>
-      <c r="E3" t="str">
+      <c r="F3" t="str">
         <v>TEMU1234567</v>
       </c>
-      <c r="F3" t="str">
+      <c r="G3" t="str">
         <v>40HC</v>
       </c>
-      <c r="G3" t="str">
+      <c r="H3" t="str">
         <v>SEAL001</v>
       </c>
-      <c r="H3" t="str">
+      <c r="I3" t="str">
         <v>BL12345678</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I3"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>